<commit_message>
Restart cycle-2 week numbering at W1 (Aug 3) across schedule, app, workbooks
Per Joe: the relaunched routes read as Week 1, not Week 3. Cycle 2 is now
W1-W9 (Aug 3 -> Sep 28) in the schedule CSV, the app week chips, the MMC
import labels, and every PL workbook's Weekly Plan tab. The executed
Jul 22-31 rows are preserved as C1-W1/C1-W2 so nothing collides. Stop
placement is unchanged - labels only.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ei2NMkxuP1dquQsjedq4wC
</commit_message>
<xml_diff>
--- a/pm/route-days-v2/Spine-Route-Days-Coty.xlsx
+++ b/pm/route-days-v2/Spine-Route-Days-Coty.xlsx
@@ -608,7 +608,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Passed in W1/W2 — revisit rotation</t>
+          <t>Passed in cycle 1 (Jul 22–31) — revisit rotation</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>Passed in W1/W2 — revisit rotation</t>
+          <t>Passed in cycle 1 (Jul 22–31) — revisit rotation</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>Passed in W1/W2 — revisit rotation</t>
+          <t>Passed in cycle 1 (Jul 22–31) — revisit rotation</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Passed in W1/W2 — revisit rotation</t>
+          <t>Passed in cycle 1 (Jul 22–31) — revisit rotation</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Passed in W1/W2 — revisit rotation</t>
+          <t>Passed in cycle 1 (Jul 22–31) — revisit rotation</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -17987,7 +17987,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -18017,7 +18017,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -18047,7 +18047,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -18077,7 +18077,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -18107,7 +18107,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -18137,7 +18137,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -18167,7 +18167,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -18197,7 +18197,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -18227,7 +18227,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -18257,7 +18257,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -18287,7 +18287,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -18317,7 +18317,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -18347,7 +18347,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -18377,7 +18377,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -18407,7 +18407,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -18437,7 +18437,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -18467,7 +18467,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W3</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -18497,7 +18497,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -18527,7 +18527,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -18557,7 +18557,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -18587,7 +18587,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -18617,7 +18617,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -18647,7 +18647,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -18677,7 +18677,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -18707,7 +18707,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -18737,7 +18737,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -18767,7 +18767,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -18797,7 +18797,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -18827,7 +18827,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -18857,7 +18857,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -18887,7 +18887,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -18917,7 +18917,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -18947,7 +18947,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -18977,7 +18977,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>W7</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -19007,7 +19007,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -19037,7 +19037,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -19067,7 +19067,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -19097,7 +19097,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -19127,7 +19127,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -19157,7 +19157,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -19187,7 +19187,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -19217,7 +19217,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>W8</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -19247,7 +19247,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -19277,7 +19277,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -19307,7 +19307,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -19337,7 +19337,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -19367,7 +19367,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -19397,7 +19397,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -19427,7 +19427,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -19457,7 +19457,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -19487,7 +19487,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -19517,7 +19517,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -19547,7 +19547,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -19577,7 +19577,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -19607,7 +19607,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>W9</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -19637,7 +19637,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -19667,7 +19667,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -19697,7 +19697,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -19727,7 +19727,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -19757,7 +19757,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -19787,7 +19787,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -19817,7 +19817,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -19847,7 +19847,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -19877,7 +19877,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -19907,7 +19907,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>W10</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -19937,7 +19937,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -19967,7 +19967,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -19997,7 +19997,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -20027,7 +20027,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -20057,7 +20057,7 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -20087,7 +20087,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -20117,7 +20117,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -20147,7 +20147,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -20177,7 +20177,7 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>W11</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">

</xml_diff>